<commit_message>
Add exploratory test reports and evidence screenshots
</commit_message>
<xml_diff>
--- a/docs/exploratory-test-report.xlsx
+++ b/docs/exploratory-test-report.xlsx
@@ -15,12 +15,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="141">
   <si>
     <t>Exploratory Test Report Summary</t>
   </si>
   <si>
-    <t>Manual report template prepared for PITON study-case delivery.</t>
+    <t>Manual exploratory observations updated from real execution results.</t>
   </si>
   <si>
     <t>Section</t>
@@ -35,19 +35,55 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Exploratory Testing Scope</t>
+    <t>DemoQA automation</t>
+  </si>
+  <si>
+    <t>https://demoqa.com/</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>15 Playwright tests passed for Elements, Forms, and Widgets modules.</t>
+  </si>
+  <si>
+    <t>PITON manual test</t>
+  </si>
+  <si>
+    <t>https://piton.com.tr/</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>2 low severity UI/responsive issues found. Navigation, footer, form validation, and Chrome/Edge visual checks passed.</t>
+  </si>
+  <si>
+    <t>GNS Metal manual test</t>
   </si>
   <si>
     <t>https://www.gnsmetal.com/home</t>
   </si>
   <si>
-    <t>To be executed manually</t>
-  </si>
-  <si>
-    <t>Capture usability, navigation, validation, visual, responsive, and performance observations.</t>
-  </si>
-  <si>
-    <t>https://piton.com.tr/</t>
+    <t>No critical issue observed in the tested scope. Contact form validation is Not Applicable because no standard user-fillable contact form was identified.</t>
+  </si>
+  <si>
+    <t>Browsers checked</t>
+  </si>
+  <si>
+    <t>Chrome and Edge</t>
+  </si>
+  <si>
+    <t>Cross-browser visual checks looked consistent for both PITON and GNS Metal in tested scope.</t>
+  </si>
+  <si>
+    <t>Viewports checked</t>
+  </si>
+  <si>
+    <t>Desktop, mobile, Galaxy Z Fold 5 responsive view</t>
+  </si>
+  <si>
+    <t>PITON Galaxy Z Fold 5 responsive view has a low severity hero text clipping issue. Other checked responsive views were generally working correctly.</t>
   </si>
   <si>
     <t>Evidence</t>
@@ -56,13 +92,13 @@
     <t>docs/screenshots/</t>
   </si>
   <si>
-    <t>Attach screenshots or video references for defects and notable observations.</t>
+    <t>Evidence screenshots for open PITON issues are stored under docs/screenshots/.</t>
   </si>
   <si>
     <t>GNS Metal Findings</t>
   </si>
   <si>
-    <t>Manual exploratory findings template.</t>
+    <t>Manual exploratory findings from tested scope.</t>
   </si>
   <si>
     <t>Bug ID</t>
@@ -101,79 +137,226 @@
     <t>Evidence/Screenshot</t>
   </si>
   <si>
-    <t>GNS-001</t>
+    <t>GNS-NAV-001</t>
   </si>
   <si>
     <t>GNS Metal</t>
   </si>
   <si>
-    <t>Home page</t>
-  </si>
-  <si>
-    <t>UX and usability</t>
-  </si>
-  <si>
-    <t>Placeholder for manual exploratory observation.</t>
-  </si>
-  <si>
-    <t>Open the website; review primary content, calls to action, and readability.</t>
-  </si>
-  <si>
-    <t>User can understand the page purpose and continue without confusion.</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>GNS-002</t>
-  </si>
-  <si>
-    <t>Navigation</t>
+    <t>Header menu</t>
   </si>
   <si>
     <t>Navigation flow</t>
   </si>
   <si>
-    <t>Placeholder for broken or confusing navigation paths.</t>
-  </si>
-  <si>
-    <t>Use header, footer, and key internal links.</t>
-  </si>
-  <si>
-    <t>Navigation works consistently and leads to expected pages.</t>
-  </si>
-  <si>
-    <t>GNS-003</t>
-  </si>
-  <si>
-    <t>Forms / Contact areas</t>
+    <t>Header/menu navigation links checked.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website and click header/menu navigation links.</t>
+  </si>
+  <si>
+    <t>Navigation links open the expected pages or sections.</t>
+  </si>
+  <si>
+    <t>Header/menu navigation links work correctly.</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>GNS-FOOT-001</t>
+  </si>
+  <si>
+    <t>Footer</t>
+  </si>
+  <si>
+    <t>Footer links checked.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website and click footer links.</t>
+  </si>
+  <si>
+    <t>Footer links open the expected destinations.</t>
+  </si>
+  <si>
+    <t>Footer links work correctly.</t>
+  </si>
+  <si>
+    <t>GNS-RESP-001</t>
+  </si>
+  <si>
+    <t>Responsive layout</t>
+  </si>
+  <si>
+    <t>Responsive behavior</t>
+  </si>
+  <si>
+    <t>Responsive layout checked.</t>
+  </si>
+  <si>
+    <t>Open the website in checked responsive viewports and inspect layout.</t>
+  </si>
+  <si>
+    <t>Layout adapts without major visual or usability issues.</t>
+  </si>
+  <si>
+    <t>Responsive layout was checked and no major visual issue was observed.</t>
+  </si>
+  <si>
+    <t>GNS-COMPAT-001</t>
+  </si>
+  <si>
+    <t>General visual layout</t>
+  </si>
+  <si>
+    <t>Browser compatibility</t>
+  </si>
+  <si>
+    <t>Chrome and Edge compatibility checked.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website in Chrome and Edge and compare main visual layout.</t>
+  </si>
+  <si>
+    <t>Visual layout is consistent across checked browsers.</t>
+  </si>
+  <si>
+    <t>Chrome and Edge visual checks look consistent.</t>
+  </si>
+  <si>
+    <t>GNS-FORM-001</t>
+  </si>
+  <si>
+    <t>Contact form</t>
   </si>
   <si>
     <t>Form validation</t>
   </si>
   <si>
-    <t>Placeholder for required field, invalid format, and submission validation findings.</t>
-  </si>
-  <si>
-    <t>Submit forms with empty and invalid values, then with valid values if available.</t>
-  </si>
-  <si>
-    <t>Validation messages are clear and invalid submissions are prevented.</t>
+    <t>Contact form validation testing.</t>
+  </si>
+  <si>
+    <t>Search tested scope for a standard user-fillable contact form.</t>
+  </si>
+  <si>
+    <t>If a user-fillable contact form exists, required field and invalid input validation can be tested.</t>
+  </si>
+  <si>
+    <t>Not Applicable because no standard user-fillable contact form was identified in the tested scope.</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
   </si>
   <si>
     <t>PITON Findings</t>
   </si>
   <si>
-    <t>PITON-001</t>
+    <t>PITON-NAV-001</t>
   </si>
   <si>
     <t>PITON</t>
   </si>
   <si>
-    <t>PITON-002</t>
-  </si>
-  <si>
-    <t>PITON-003</t>
+    <t>Open PITON website and click header/menu navigation links.</t>
+  </si>
+  <si>
+    <t>PITON-FOOT-001</t>
+  </si>
+  <si>
+    <t>Open PITON website and click footer links.</t>
+  </si>
+  <si>
+    <t>PITON-FORM-001</t>
+  </si>
+  <si>
+    <t>Empty submit validation checked.</t>
+  </si>
+  <si>
+    <t>Open contact form and submit without filling required fields.</t>
+  </si>
+  <si>
+    <t>Required field warnings are displayed and empty submission is prevented.</t>
+  </si>
+  <si>
+    <t>Contact form warns the user when required fields are empty.</t>
+  </si>
+  <si>
+    <t>PITON-FORM-002</t>
+  </si>
+  <si>
+    <t>Contact form email field</t>
+  </si>
+  <si>
+    <t>Invalid email validation checked.</t>
+  </si>
+  <si>
+    <t>Enter an invalid email value without @ and submit the contact form.</t>
+  </si>
+  <si>
+    <t>Email field displays a clear invalid email warning.</t>
+  </si>
+  <si>
+    <t>Email field warns the user that an @ character is required.</t>
+  </si>
+  <si>
+    <t>PITON-COMPAT-001</t>
+  </si>
+  <si>
+    <t>Open PITON website in Chrome and Edge and compare main visual layout.</t>
+  </si>
+  <si>
+    <t>PITON-UI-001</t>
+  </si>
+  <si>
+    <t>Contact form subject dropdown</t>
+  </si>
+  <si>
+    <t>Visual/UI consistency</t>
+  </si>
+  <si>
+    <t>Contact form subject dropdown visual contrast/theme inconsistency.</t>
+  </si>
+  <si>
+    <t>Open the contact form and expand the Konu dropdown.</t>
+  </si>
+  <si>
+    <t>Dropdown option area follows the site dark theme and remains readable.</t>
+  </si>
+  <si>
+    <t>Dropdown option area appears as a large white/blank area, creating visual consistency and contrast problems.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>docs/screenshots/piton-contact-subject-dropdown-contrast-issue.png</t>
+  </si>
+  <si>
+    <t>PITON-RESP-001</t>
+  </si>
+  <si>
+    <t>Homepage hero</t>
+  </si>
+  <si>
+    <t>Homepage hero text clipping on Galaxy Z Fold 5 responsive view.</t>
+  </si>
+  <si>
+    <t>Open PITON homepage in Galaxy Z Fold 5 responsive viewport and inspect hero text.</t>
+  </si>
+  <si>
+    <t>Hero text should be fully visible without clipping.</t>
+  </si>
+  <si>
+    <t>A small part of the homepage hero text is clipped/not fully visible.</t>
+  </si>
+  <si>
+    <t>docs/screenshots/piton-home-galaxy-z-fold-text-clipping.png</t>
   </si>
   <si>
     <t>Browser Compatibility</t>
@@ -197,16 +380,16 @@
     <t>Chrome</t>
   </si>
   <si>
+    <t>Manual check</t>
+  </si>
+  <si>
     <t>Home and key navigation pages</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Firefox</t>
-  </si>
-  <si>
-    <t>Safari / WebKit</t>
+    <t>Visual checks look consistent.</t>
+  </si>
+  <si>
+    <t>Edge</t>
   </si>
   <si>
     <t>Responsive Checks</t>
@@ -230,35 +413,38 @@
     <t>Desktop</t>
   </si>
   <si>
-    <t>1440x900</t>
-  </si>
-  <si>
     <t>Header, hero, navigation, footer</t>
   </si>
   <si>
-    <t>Tablet</t>
-  </si>
-  <si>
-    <t>768x1024</t>
-  </si>
-  <si>
-    <t>Header, content layout, forms</t>
+    <t>No major visual issue observed.</t>
   </si>
   <si>
     <t>Mobile</t>
   </si>
   <si>
-    <t>390x844</t>
-  </si>
-  <si>
-    <t>Menu, content stacking, forms</t>
+    <t>Menu, content stacking, key pages</t>
+  </si>
+  <si>
+    <t>Generally working correctly.</t>
+  </si>
+  <si>
+    <t>Menu, content stacking, contact form</t>
+  </si>
+  <si>
+    <t>Galaxy Z Fold 5</t>
+  </si>
+  <si>
+    <t>Responsive viewport</t>
+  </si>
+  <si>
+    <t>A small part of hero text is clipped/not fully visible.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -281,10 +467,18 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF006100"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF9C0006"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF666666"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -298,7 +492,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -344,7 +548,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -357,6 +561,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -698,7 +908,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -753,30 +963,72 @@
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -792,7 +1044,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -809,7 +1061,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -825,7 +1077,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -841,154 +1093,230 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>28</v>
+        <v>40</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>47</v>
+        <v>61</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -1004,7 +1332,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1021,7 +1349,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>78</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1037,7 +1365,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1053,154 +1381,306 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>27</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>49</v>
+        <v>79</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="D5" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>8</v>
+        <v>55</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>43</v>
+        <v>71</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>44</v>
+        <v>72</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>46</v>
+        <v>86</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>8</v>
+        <v>88</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="L6" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="K9" s="6" t="s">
         <v>12</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="K10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1216,7 +1696,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1228,7 +1708,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>53</v>
+        <v>114</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1238,7 +1718,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>54</v>
+        <v>115</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1248,19 +1728,19 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>55</v>
+        <v>116</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>56</v>
+        <v>117</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>57</v>
+        <v>118</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>58</v>
+        <v>119</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>5</v>
@@ -1268,122 +1748,82 @@
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>59</v>
+        <v>120</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>35</v>
+        <v>121</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E4" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>62</v>
+        <v>124</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>35</v>
+        <v>121</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E5" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>35</v>
+        <v>121</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>59</v>
+        <v>124</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>35</v>
+        <v>121</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E7" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -1399,7 +1839,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1412,7 +1852,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>64</v>
+        <v>125</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1423,7 +1863,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>65</v>
+        <v>126</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1434,163 +1874,140 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>66</v>
+        <v>127</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>67</v>
+        <v>128</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>68</v>
+        <v>129</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>69</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>72</v>
+        <v>132</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>73</v>
+        <v>134</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>74</v>
+        <v>121</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>75</v>
+        <v>135</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>8</v>
+        <v>133</v>
       </c>
       <c r="F5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>29</v>
+        <v>80</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>78</v>
+        <v>132</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>8</v>
+        <v>136</v>
       </c>
       <c r="F6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>70</v>
+        <v>134</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>72</v>
+        <v>137</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>8</v>
+        <v>136</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>73</v>
+        <v>138</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>74</v>
+        <v>139</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>8</v>
+        <v>140</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>12</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>12</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add GNS products page performance observation
</commit_message>
<xml_diff>
--- a/docs/exploratory-test-report.xlsx
+++ b/docs/exploratory-test-report.xlsx
@@ -15,75 +15,126 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="230">
   <si>
     <t>Exploratory Test Report Summary</t>
   </si>
   <si>
-    <t>Manual exploratory observations updated from real execution results.</t>
-  </si>
-  <si>
-    <t>Section</t>
-  </si>
-  <si>
-    <t>Website / Scope</t>
-  </si>
-  <si>
-    <t>Current Status</t>
+    <t>Manual exploratory observations based on real execution results.</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Status / Value</t>
   </si>
   <si>
     <t>Notes</t>
   </si>
   <si>
+    <t>Project name</t>
+  </si>
+  <si>
+    <t>PITON &amp; GNS Web Test</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Manual exploratory testing deliverable for corporate websites, alongside DemoQA automation.</t>
+  </si>
+  <si>
+    <t>Test type</t>
+  </si>
+  <si>
+    <t>Manual Exploratory Testing</t>
+  </si>
+  <si>
+    <t>Corporate websites were tested manually, not automated.</t>
+  </si>
+  <si>
+    <t>Website tested</t>
+  </si>
+  <si>
+    <t>https://www.gnsmetal.com/home</t>
+  </si>
+  <si>
+    <t>GNS Metal website tested in the documented scope.</t>
+  </si>
+  <si>
+    <t>https://piton.com.tr/</t>
+  </si>
+  <si>
+    <t>PITON website tested in the documented scope.</t>
+  </si>
+  <si>
+    <t>Browsers checked</t>
+  </si>
+  <si>
+    <t>Chrome, Edge</t>
+  </si>
+  <si>
+    <t>Passed</t>
+  </si>
+  <si>
+    <t>No major browser-specific rendering difference was observed in the tested scope.</t>
+  </si>
+  <si>
+    <t>Viewports checked</t>
+  </si>
+  <si>
+    <t>Desktop, Tablet, Mobile, Galaxy Z Fold 5 responsive view</t>
+  </si>
+  <si>
+    <t>Open</t>
+  </si>
+  <si>
+    <t>PITON Galaxy Z Fold 5 responsive view has a low severity hero text clipping issue.</t>
+  </si>
+  <si>
+    <t>Automation note</t>
+  </si>
+  <si>
+    <t>Corporate websites</t>
+  </si>
+  <si>
+    <t>Not Applicable</t>
+  </si>
+  <si>
+    <t>No automation was written for corporate websites, in accordance with the study-case requirement.</t>
+  </si>
+  <si>
     <t>DemoQA automation</t>
   </si>
   <si>
     <t>https://demoqa.com/</t>
   </si>
   <si>
-    <t>Passed</t>
-  </si>
-  <si>
     <t>15 Playwright tests passed for Elements, Forms, and Widgets modules.</t>
   </si>
   <si>
-    <t>PITON manual test</t>
-  </si>
-  <si>
-    <t>https://piton.com.tr/</t>
-  </si>
-  <si>
-    <t>Open</t>
-  </si>
-  <si>
-    <t>2 low severity UI/responsive issues found. Navigation, footer, form validation, and Chrome/Edge visual checks passed.</t>
-  </si>
-  <si>
-    <t>GNS Metal manual test</t>
-  </si>
-  <si>
-    <t>https://www.gnsmetal.com/home</t>
-  </si>
-  <si>
-    <t>No critical issue observed in the tested scope. Contact form validation is Not Applicable because no standard user-fillable contact form was identified.</t>
-  </si>
-  <si>
-    <t>Browsers checked</t>
-  </si>
-  <si>
-    <t>Chrome and Edge</t>
-  </si>
-  <si>
-    <t>Cross-browser visual checks looked consistent for both PITON and GNS Metal in tested scope.</t>
-  </si>
-  <si>
-    <t>Viewports checked</t>
-  </si>
-  <si>
-    <t>Desktop, mobile, Galaxy Z Fold 5 responsive view</t>
-  </si>
-  <si>
-    <t>PITON Galaxy Z Fold 5 responsive view has a low severity hero text clipping issue. Other checked responsive views were generally working correctly.</t>
+    <t>PITON summary counts</t>
+  </si>
+  <si>
+    <t>Passed checks: 11; Open issues: 2</t>
+  </si>
+  <si>
+    <t>PITON has two low-severity UI/responsive findings.</t>
+  </si>
+  <si>
+    <t>GNS Metal summary counts</t>
+  </si>
+  <si>
+    <t>Passed checks: 9; Not Applicable checks: 1; Observations: 1; Open issues: 0</t>
+  </si>
+  <si>
+    <t>Observation</t>
+  </si>
+  <si>
+    <t>GNS Metal had one low-severity page loading observation and no critical functional issue observed in the tested scope.</t>
   </si>
   <si>
     <t>Evidence</t>
@@ -95,13 +146,22 @@
     <t>Evidence screenshots for open PITON issues are stored under docs/screenshots/.</t>
   </si>
   <si>
+    <t>Brief conclusion</t>
+  </si>
+  <si>
+    <t>Manual exploratory result</t>
+  </si>
+  <si>
+    <t>PITON has two low-severity UI/responsive findings. GNS Metal has one low-severity page loading observation and no critical functional issue observed in the tested scope.</t>
+  </si>
+  <si>
     <t>GNS Metal Findings</t>
   </si>
   <si>
     <t>Manual exploratory findings from tested scope.</t>
   </si>
   <si>
-    <t>Bug ID</t>
+    <t>Bug/Check ID</t>
   </si>
   <si>
     <t>Website</t>
@@ -137,12 +197,39 @@
     <t>Evidence/Screenshot</t>
   </si>
   <si>
+    <t>GNS-UX-001</t>
+  </si>
+  <si>
+    <t>GNS Metal</t>
+  </si>
+  <si>
+    <t>Homepage</t>
+  </si>
+  <si>
+    <t>UX and usability</t>
+  </si>
+  <si>
+    <t>UX and homepage usability checked.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal homepage and review main content, visual hierarchy, readability, and navigation entry points.</t>
+  </si>
+  <si>
+    <t>Homepage is understandable and usable for a first-time visitor.</t>
+  </si>
+  <si>
+    <t>No major UX/usability issue was observed in the tested scope.</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>GNS-NAV-001</t>
   </si>
   <si>
-    <t>GNS Metal</t>
-  </si>
-  <si>
     <t>Header menu</t>
   </si>
   <si>
@@ -161,12 +248,6 @@
     <t>Header/menu navigation links work correctly.</t>
   </si>
   <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>GNS-FOOT-001</t>
   </si>
   <si>
@@ -185,28 +266,109 @@
     <t>Footer links work correctly.</t>
   </si>
   <si>
+    <t>GNS-LINK-001</t>
+  </si>
+  <si>
+    <t>Tested navigation scope</t>
+  </si>
+  <si>
+    <t>Broken links</t>
+  </si>
+  <si>
+    <t>Broken link observation in tested navigation scope.</t>
+  </si>
+  <si>
+    <t>Use header/menu and footer links during exploratory navigation.</t>
+  </si>
+  <si>
+    <t>Checked links should navigate successfully without obvious broken-link behavior.</t>
+  </si>
+  <si>
+    <t>No broken link behavior was observed in the tested navigation scope.</t>
+  </si>
+  <si>
+    <t>GNS-FORM-001</t>
+  </si>
+  <si>
+    <t>Contact form</t>
+  </si>
+  <si>
+    <t>Form validation</t>
+  </si>
+  <si>
+    <t>Contact form validation testing.</t>
+  </si>
+  <si>
+    <t>Search tested scope for a standard user-fillable contact form.</t>
+  </si>
+  <si>
+    <t>If a user-fillable contact form exists, required field and invalid input validation can be tested.</t>
+  </si>
+  <si>
+    <t>Not Applicable because no standard user-fillable contact form was identified in the tested scope.</t>
+  </si>
+  <si>
+    <t>GNS-UI-001</t>
+  </si>
+  <si>
+    <t>General pages</t>
+  </si>
+  <si>
+    <t>Visual/UI consistency</t>
+  </si>
+  <si>
+    <t>Visual/UI consistency checked.</t>
+  </si>
+  <si>
+    <t>Review tested GNS Metal pages for obvious layout, spacing, typography, and color consistency issues.</t>
+  </si>
+  <si>
+    <t>No major visual consistency issue is observed.</t>
+  </si>
+  <si>
+    <t>No major visual/UI consistency issue was observed in the tested scope.</t>
+  </si>
+  <si>
     <t>GNS-RESP-001</t>
   </si>
   <si>
-    <t>Responsive layout</t>
+    <t>Desktop layout</t>
   </si>
   <si>
     <t>Responsive behavior</t>
   </si>
   <si>
-    <t>Responsive layout checked.</t>
-  </si>
-  <si>
-    <t>Open the website in checked responsive viewports and inspect layout.</t>
+    <t>Responsive desktop check.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website in desktop viewport and inspect main sections.</t>
+  </si>
+  <si>
+    <t>Layout is readable and usable on desktop.</t>
+  </si>
+  <si>
+    <t>Desktop responsive layout was checked and no major visual issue was observed.</t>
+  </si>
+  <si>
+    <t>GNS-RESP-002</t>
+  </si>
+  <si>
+    <t>Tablet/mobile layout</t>
+  </si>
+  <si>
+    <t>Responsive tablet/mobile check.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website in tablet and mobile viewports and inspect content stacking and navigation.</t>
   </si>
   <si>
     <t>Layout adapts without major visual or usability issues.</t>
   </si>
   <si>
-    <t>Responsive layout was checked and no major visual issue was observed.</t>
-  </si>
-  <si>
-    <t>GNS-COMPAT-001</t>
+    <t>Tablet/mobile responsive layout was checked and no major visual issue was observed.</t>
+  </si>
+  <si>
+    <t>GNS-COMPAT-CHROME-001</t>
   </si>
   <si>
     <t>General visual layout</t>
@@ -215,51 +377,80 @@
     <t>Browser compatibility</t>
   </si>
   <si>
-    <t>Chrome and Edge compatibility checked.</t>
-  </si>
-  <si>
-    <t>Open GNS Metal website in Chrome and Edge and compare main visual layout.</t>
-  </si>
-  <si>
-    <t>Visual layout is consistent across checked browsers.</t>
-  </si>
-  <si>
-    <t>Chrome and Edge visual checks look consistent.</t>
-  </si>
-  <si>
-    <t>GNS-FORM-001</t>
-  </si>
-  <si>
-    <t>Contact form</t>
-  </si>
-  <si>
-    <t>Form validation</t>
-  </si>
-  <si>
-    <t>Contact form validation testing.</t>
-  </si>
-  <si>
-    <t>Search tested scope for a standard user-fillable contact form.</t>
-  </si>
-  <si>
-    <t>If a user-fillable contact form exists, required field and invalid input validation can be tested.</t>
-  </si>
-  <si>
-    <t>Not Applicable because no standard user-fillable contact form was identified in the tested scope.</t>
-  </si>
-  <si>
-    <t>Not Applicable</t>
+    <t>Chrome compatibility checked.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website in Chrome and review tested pages.</t>
+  </si>
+  <si>
+    <t>No major Chrome-specific rendering issue is observed.</t>
+  </si>
+  <si>
+    <t>Chrome visual check looks consistent.</t>
+  </si>
+  <si>
+    <t>GNS-COMPAT-EDGE-001</t>
+  </si>
+  <si>
+    <t>Edge compatibility checked.</t>
+  </si>
+  <si>
+    <t>Open GNS Metal website in Edge and review tested pages.</t>
+  </si>
+  <si>
+    <t>No major Edge-specific rendering issue is observed.</t>
+  </si>
+  <si>
+    <t>Edge visual check looks consistent.</t>
+  </si>
+  <si>
+    <t>GNS-PERF-001</t>
+  </si>
+  <si>
+    <t>Ürünlerimiz page</t>
+  </si>
+  <si>
+    <t>Performance / Page Loading Observation</t>
+  </si>
+  <si>
+    <t>The Ürünlerimiz page was observed to load slower than other checked pages during manual exploratory testing. The page contains many product images and detailed content, which may contribute to the perceived loading delay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the GNS Metal website.
+2. Click the Ürünlerimiz navigation item.
+3. Compare the loading behavior with other main navigation pages.</t>
+  </si>
+  <si>
+    <t>The page should load within a reasonable time and provide a smooth navigation experience.</t>
+  </si>
+  <si>
+    <t>The Ürünlerimiz page loads slower compared to other checked pages.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>docs/screenshots/gns-products-page-loading-observation.png</t>
   </si>
   <si>
     <t>PITON Findings</t>
   </si>
   <si>
+    <t>PITON-UX-001</t>
+  </si>
+  <si>
+    <t>PITON</t>
+  </si>
+  <si>
+    <t>Open PITON homepage and review main content, visual hierarchy, readability, and primary navigation entry points.</t>
+  </si>
+  <si>
+    <t>Homepage was generally usable in the tested scope.</t>
+  </si>
+  <si>
     <t>PITON-NAV-001</t>
   </si>
   <si>
-    <t>PITON</t>
-  </si>
-  <si>
     <t>Open PITON website and click header/menu navigation links.</t>
   </si>
   <si>
@@ -302,21 +493,12 @@
     <t>Email field warns the user that an @ character is required.</t>
   </si>
   <si>
-    <t>PITON-COMPAT-001</t>
-  </si>
-  <si>
-    <t>Open PITON website in Chrome and Edge and compare main visual layout.</t>
-  </si>
-  <si>
     <t>PITON-UI-001</t>
   </si>
   <si>
     <t>Contact form subject dropdown</t>
   </si>
   <si>
-    <t>Visual/UI consistency</t>
-  </si>
-  <si>
     <t>Contact form subject dropdown visual contrast/theme inconsistency.</t>
   </si>
   <si>
@@ -329,15 +511,54 @@
     <t>Dropdown option area appears as a large white/blank area, creating visual consistency and contrast problems.</t>
   </si>
   <si>
-    <t>Low</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
     <t>docs/screenshots/piton-contact-subject-dropdown-contrast-issue.png</t>
   </si>
   <si>
+    <t>PITON-UI-002</t>
+  </si>
+  <si>
+    <t>Visual/UI consistency general check.</t>
+  </si>
+  <si>
+    <t>Review tested PITON pages for obvious layout, spacing, typography, and color consistency issues.</t>
+  </si>
+  <si>
+    <t>No major visual consistency problem is observed outside documented defects.</t>
+  </si>
+  <si>
+    <t>General visual/UI consistency looked acceptable in the tested scope, except PITON-UI-001.</t>
+  </si>
+  <si>
+    <t>PITON-RESP-002</t>
+  </si>
+  <si>
+    <t>Open PITON website in desktop viewport and inspect main sections.</t>
+  </si>
+  <si>
+    <t>Desktop view worked correctly in the tested scope.</t>
+  </si>
+  <si>
+    <t>PITON-RESP-003</t>
+  </si>
+  <si>
+    <t>Mobile layout</t>
+  </si>
+  <si>
+    <t>Responsive mobile check.</t>
+  </si>
+  <si>
+    <t>Open PITON website in mobile viewport and inspect navigation, content stacking, and contact form areas.</t>
+  </si>
+  <si>
+    <t>Mobile layout is readable and usable.</t>
+  </si>
+  <si>
+    <t>Mobile view generally works correctly.</t>
+  </si>
+  <si>
     <t>PITON-RESP-001</t>
   </si>
   <si>
@@ -359,6 +580,39 @@
     <t>docs/screenshots/piton-home-galaxy-z-fold-text-clipping.png</t>
   </si>
   <si>
+    <t>PITON-COMPAT-CHROME-001</t>
+  </si>
+  <si>
+    <t>Open PITON website in Chrome and review tested pages.</t>
+  </si>
+  <si>
+    <t>PITON-COMPAT-EDGE-001</t>
+  </si>
+  <si>
+    <t>Open PITON website in Edge and review tested pages.</t>
+  </si>
+  <si>
+    <t>PITON-PERF-001</t>
+  </si>
+  <si>
+    <t>General page loading</t>
+  </si>
+  <si>
+    <t>Performance observation</t>
+  </si>
+  <si>
+    <t>Basic page loading observation.</t>
+  </si>
+  <si>
+    <t>Open PITON website and observe whether tested pages load without obvious blocking or broken content.</t>
+  </si>
+  <si>
+    <t>Pages load sufficiently for manual exploration without obvious blocking issues.</t>
+  </si>
+  <si>
+    <t>No major page loading issue was observed during manual checks.</t>
+  </si>
+  <si>
     <t>Browser Compatibility</t>
   </si>
   <si>
@@ -368,7 +622,7 @@
     <t>Browser</t>
   </si>
   <si>
-    <t>Version</t>
+    <t>Viewport</t>
   </si>
   <si>
     <t>Primary Pages Checked</t>
@@ -380,37 +634,67 @@
     <t>Chrome</t>
   </si>
   <si>
+    <t>Desktop</t>
+  </si>
+  <si>
+    <t>Home, navigation, footer, contact form</t>
+  </si>
+  <si>
+    <t>No major browser-specific rendering difference was observed.</t>
+  </si>
+  <si>
+    <t>Edge</t>
+  </si>
+  <si>
+    <t>Home and key navigation pages</t>
+  </si>
+  <si>
+    <t>Responsive Checks</t>
+  </si>
+  <si>
+    <t>Manual responsive behavior checklist.</t>
+  </si>
+  <si>
+    <t>Resolution</t>
+  </si>
+  <si>
+    <t>Areas Checked</t>
+  </si>
+  <si>
+    <t>Notes / Evidence</t>
+  </si>
+  <si>
     <t>Manual check</t>
   </si>
   <si>
-    <t>Home and key navigation pages</t>
-  </si>
-  <si>
-    <t>Visual checks look consistent.</t>
-  </si>
-  <si>
-    <t>Edge</t>
-  </si>
-  <si>
-    <t>Responsive Checks</t>
-  </si>
-  <si>
-    <t>Manual responsive behavior checklist.</t>
-  </si>
-  <si>
-    <t>Viewport</t>
-  </si>
-  <si>
-    <t>Resolution</t>
-  </si>
-  <si>
-    <t>Areas Checked</t>
-  </si>
-  <si>
-    <t>Notes / Evidence</t>
-  </si>
-  <si>
-    <t>Desktop</t>
+    <t>Header, hero, navigation, footer, contact form</t>
+  </si>
+  <si>
+    <t>Tablet</t>
+  </si>
+  <si>
+    <t>Navigation, content stacking, contact form</t>
+  </si>
+  <si>
+    <t>Tablet view was checked with no major visual issue observed.</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Menu, content stacking, contact form</t>
+  </si>
+  <si>
+    <t>Galaxy Z Fold 5</t>
+  </si>
+  <si>
+    <t>Responsive viewport</t>
+  </si>
+  <si>
+    <t>A small part of hero text is clipped/not fully visible.</t>
+  </si>
+  <si>
+    <t>PITON-RESP-001; docs/screenshots/piton-home-galaxy-z-fold-text-clipping.png</t>
   </si>
   <si>
     <t>Header, hero, navigation, footer</t>
@@ -419,32 +703,17 @@
     <t>No major visual issue observed.</t>
   </si>
   <si>
-    <t>Mobile</t>
+    <t>Header, content layout, navigation, footer</t>
   </si>
   <si>
     <t>Menu, content stacking, key pages</t>
-  </si>
-  <si>
-    <t>Generally working correctly.</t>
-  </si>
-  <si>
-    <t>Menu, content stacking, contact form</t>
-  </si>
-  <si>
-    <t>Galaxy Z Fold 5</t>
-  </si>
-  <si>
-    <t>Responsive viewport</t>
-  </si>
-  <si>
-    <t>A small part of hero text is clipped/not fully visible.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -477,8 +746,12 @@
       <b/>
       <color rgb="FF666666"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF9C6500"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -503,6 +776,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -548,7 +826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -567,6 +845,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -908,13 +1189,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
     <col min="3" max="3" width="32" customWidth="1"/>
-    <col min="4" max="4" width="55" customWidth="1"/>
+    <col min="4" max="4" width="62" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -954,7 +1235,7 @@
       <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="4" t="s">
@@ -968,67 +1249,151 @@
       <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="C9" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>8</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>25</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -1044,10 +1409,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
@@ -1061,7 +1426,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1077,7 +1442,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1093,230 +1458,458 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>56</v>
+        <v>77</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>57</v>
+        <v>78</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>60</v>
+        <v>80</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>61</v>
+        <v>81</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>62</v>
+        <v>82</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>64</v>
+        <v>84</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>68</v>
+        <v>88</v>
       </c>
       <c r="H7" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L7" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="J7" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="L7" s="4" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H8" s="4" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="L8" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="I9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L9" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1332,10 +1925,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="4" width="24" customWidth="1"/>
     <col min="5" max="5" width="42" customWidth="1"/>
@@ -1349,7 +1942,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>78</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1365,7 +1958,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1381,306 +1974,534 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>31</v>
+        <v>51</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>32</v>
+        <v>52</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>33</v>
+        <v>53</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>42</v>
+        <v>62</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>81</v>
+        <v>141</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>47</v>
+        <v>142</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K4" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>82</v>
+        <v>143</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>43</v>
+        <v>72</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>83</v>
+        <v>144</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>54</v>
+        <v>75</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>55</v>
+        <v>76</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>84</v>
+        <v>145</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>72</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>86</v>
+        <v>146</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L6" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>89</v>
+        <v>147</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>91</v>
+        <v>148</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>92</v>
+        <v>149</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>93</v>
+        <v>150</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>94</v>
+        <v>151</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="J7" s="4" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K7" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="L7" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>95</v>
+        <v>152</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>64</v>
+        <v>153</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>66</v>
+        <v>154</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>96</v>
+        <v>155</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>68</v>
+        <v>156</v>
       </c>
       <c r="H8" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L8" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="L8" s="4" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="9" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>97</v>
+        <v>158</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>98</v>
+        <v>159</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>99</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>101</v>
+        <v>161</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>102</v>
+        <v>162</v>
       </c>
       <c r="H9" s="4" t="s">
-        <v>103</v>
+        <v>163</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>104</v>
+        <v>136</v>
       </c>
       <c r="J9" s="4" t="s">
-        <v>105</v>
+        <v>164</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="L9" s="4" t="s">
-        <v>106</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="E10" s="4" t="s">
+      <c r="F11" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="G11" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="F10" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J10" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="K10" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="L10" s="4" t="s">
-        <v>113</v>
+      <c r="H11" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="I11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L11" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L12" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="K13" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="I15" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" ht="42" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>192</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -1699,16 +2520,16 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="28" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>198</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1718,7 +2539,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>115</v>
+        <v>199</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1728,19 +2549,19 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>116</v>
+        <v>200</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>117</v>
+        <v>201</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>118</v>
+        <v>202</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>119</v>
+        <v>203</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>5</v>
@@ -1748,82 +2569,82 @@
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>121</v>
+        <v>205</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>122</v>
+        <v>206</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>123</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>124</v>
+        <v>208</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>121</v>
+        <v>205</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>122</v>
+        <v>206</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>123</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>121</v>
+        <v>205</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>122</v>
+        <v>209</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>123</v>
+        <v>207</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>124</v>
+        <v>208</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>121</v>
+        <v>205</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>122</v>
+        <v>209</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>123</v>
+        <v>207</v>
       </c>
     </row>
   </sheetData>
@@ -1839,7 +2660,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -1852,7 +2673,7 @@
   <sheetData>
     <row r="1" ht="24" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>125</v>
+        <v>210</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1863,7 +2684,7 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>126</v>
+        <v>211</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1874,140 +2695,186 @@
     </row>
     <row r="3" ht="28" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>127</v>
+        <v>201</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>128</v>
+        <v>212</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>129</v>
+        <v>213</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>130</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>131</v>
+        <v>205</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>121</v>
+        <v>215</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>132</v>
+        <v>216</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>41</v>
+        <v>140</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>134</v>
+        <v>217</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>121</v>
+        <v>215</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>135</v>
+        <v>218</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>133</v>
+        <v>219</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="6" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>131</v>
+        <v>220</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>121</v>
+        <v>215</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>132</v>
+        <v>221</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>136</v>
+        <v>179</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>134</v>
+        <v>222</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>121</v>
+        <v>223</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>137</v>
+        <v>181</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>8</v>
+        <v>224</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>24</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>49</v>
+        <v>225</v>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>138</v>
+        <v>205</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>139</v>
+        <v>215</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>108</v>
+        <v>226</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>12</v>
+        <v>227</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>113</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>